<commit_message>
Add new Excel files and update existing ones in isSent directory
- Added new Excel files: dd.xlsx and dd_2.xlsx
- Updated existing Excel file: telegram_emails.xlsx
</commit_message>
<xml_diff>
--- a/isSent/telegram_emails.xlsx
+++ b/isSent/telegram_emails.xlsx
@@ -24,63 +24,27 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>Email</t>
   </si>
   <si>
-    <t>𝐛𝐚𝐧𝐢𝐤𝐚.𝐰𝐚𝐳𝐢𝐫@𝐩𝐫𝐨𝐠𝐫𝐚𝐦𝐦𝐢𝐧𝐠.𝐜𝐨𝐦</t>
-  </si>
-  <si>
-    <t>adil@intineriinfosol.com</t>
-  </si>
-  <si>
-    <t>Jayalakshmi@etek.solutions</t>
-  </si>
-  <si>
-    <t>navya_sethi@technologymindz.com</t>
-  </si>
-  <si>
-    <t>manjula_jakkula@epam.com</t>
-  </si>
-  <si>
-    <t>udayasri.m@martinettechnologies.com</t>
-  </si>
-  <si>
-    <t>hr@aipxperts.com</t>
-  </si>
-  <si>
-    <t>sayantan-dutta@hcltech.com</t>
-  </si>
-  <si>
-    <t>mamta.yadav@firminiq.com</t>
-  </si>
-  <si>
-    <t>jayti.agarwal@qtsolv.com</t>
-  </si>
-  <si>
-    <t>megha.ns@eastencher.com</t>
-  </si>
-  <si>
-    <t>jai.pannerselvam@perficient.com</t>
-  </si>
-  <si>
-    <t>kritika.dhar@capgemini.com</t>
-  </si>
-  <si>
-    <t>Yamini@blockstack.tech</t>
-  </si>
-  <si>
-    <t>rasik.jidewar@telomeregs.com</t>
-  </si>
-  <si>
-    <t>sainavitha@deltacubes.us</t>
-  </si>
-  <si>
-    <t>da@asanlabs.com</t>
-  </si>
-  <si>
-    <t>Grace.Yosephine@rsystems.com</t>
+    <t>nikita@insuredmine.com</t>
+  </si>
+  <si>
+    <t>rohan@insuredmine.com</t>
+  </si>
+  <si>
+    <t>recruitment@atdrive.com</t>
+  </si>
+  <si>
+    <t>𝐚𝐧𝐮𝐯𝐚@𝐡𝐢𝐧𝐝𝐮𝐬𝐭𝐚𝐧𝐭𝐢𝐦𝐞𝐬.𝐜𝐨𝐦</t>
+  </si>
+  <si>
+    <t>riya.hiwarale@alphacom.in</t>
+  </si>
+  <si>
+    <t>devayani.r@kamlaxglobal.com</t>
   </si>
 </sst>
 </file>
@@ -125,9 +89,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -436,7 +401,7 @@
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
     </row>
@@ -451,86 +416,50 @@
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A8" s="1" t="s">
-        <v>7</v>
-      </c>
+      <c r="A8" s="1"/>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A9" s="1" t="s">
-        <v>8</v>
-      </c>
+      <c r="A9" s="1"/>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A10" s="1" t="s">
-        <v>9</v>
-      </c>
+      <c r="A10" s="1"/>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A11" s="1" t="s">
-        <v>10</v>
-      </c>
+      <c r="A11" s="1"/>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A12" s="1" t="s">
-        <v>11</v>
-      </c>
+      <c r="A12" s="1"/>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A13" s="1" t="s">
-        <v>12</v>
-      </c>
+      <c r="A13" s="1"/>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A14" s="1" t="s">
-        <v>13</v>
-      </c>
+      <c r="A14" s="1"/>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A15" s="1" t="s">
-        <v>14</v>
-      </c>
+      <c r="A15" s="1"/>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A16" s="1" t="s">
-        <v>15</v>
-      </c>
+      <c r="A16" s="1"/>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A17" s="1" t="s">
-        <v>16</v>
-      </c>
+      <c r="A17" s="1"/>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A18" s="1" t="s">
-        <v>17</v>
-      </c>
+      <c r="A18" s="1"/>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A19" s="1" t="s">
-        <v>18</v>
-      </c>
+      <c r="A19" s="1"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A3" r:id="rId1" display="mailto:adil@intineriinfosol.com"/>
-    <hyperlink ref="A4" r:id="rId2" display="https://Jayalakshmi@etek.solutions/"/>
-    <hyperlink ref="A5" r:id="rId3" display="mailto:navya_sethi@technologymindz.com"/>
-    <hyperlink ref="A6" r:id="rId4" display="mailto:manjula_jakkula@epam.com"/>
-    <hyperlink ref="A7" r:id="rId5" display="mailto:udayasri.m@martinettechnologies.com"/>
-    <hyperlink ref="A8" r:id="rId6" display="mailto:hr@aipxperts.com"/>
-    <hyperlink ref="A9" r:id="rId7" display="mailto:sayantan-dutta@hcltech.com"/>
-    <hyperlink ref="A10" r:id="rId8" display="mailto:mamta.yadav@firminiq.com"/>
-    <hyperlink ref="A11" r:id="rId9" display="mailto:jayti.agarwal@qtsolv.com"/>
-    <hyperlink ref="A12" r:id="rId10" display="mailto:megha.ns@eastencher.com"/>
-    <hyperlink ref="A13" r:id="rId11" display="mailto:jai.pannerselvam@perficient.com"/>
-    <hyperlink ref="A14" r:id="rId12" display="mailto:kritika.dhar@capgemini.com"/>
-    <hyperlink ref="A15" r:id="rId13" display="mailto:Yamini@blockstack.tech"/>
-    <hyperlink ref="A16" r:id="rId14" display="mailto:rasik.jidewar@telomeregs.com"/>
-    <hyperlink ref="A17" r:id="rId15" display="mailto:sainavitha@deltacubes.us"/>
-    <hyperlink ref="A18" r:id="rId16" display="mailto:da@asanlabs.com"/>
-    <hyperlink ref="A19" r:id="rId17" display="mailto:Grace.Yosephine@rsystems.com"/>
+    <hyperlink ref="A2" r:id="rId1" display="mailto:nikita@insuredmine.com"/>
+    <hyperlink ref="A3" r:id="rId2" display="mailto:rohan@insuredmine.com"/>
+    <hyperlink ref="A4" r:id="rId3" display="mailto:recruitment@atdrive.com"/>
+    <hyperlink ref="A6" r:id="rId4" display="mailto:riya.hiwarale@alphacom.in"/>
+    <hyperlink ref="A7" r:id="rId5" display="mailto:devayani.r@kamlaxglobal.com"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId18"/>
+  <pageSetup orientation="portrait" r:id="rId6"/>
 </worksheet>
 </file>
</xml_diff>